<commit_message>
Update BOC USD rates (auto)
</commit_message>
<xml_diff>
--- a/data/2026/2026-09.xlsx
+++ b/data/2026/2026-09.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Daily Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Published Values'!$A$1:$J$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Published Values'!$A$1:$J$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Daily Summary'!$A$1:$E$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4188,8 +4188,60 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-09-13 05:30:00</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>669.74</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>669.74</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>672.55</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>672.55</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>677.43</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>2026/09/13 05:30:00</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-09-12 22:15:12</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://www.bankofchina.com/sourcedb/whpj/enindex_1619.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J72"/>
+  <autoFilter ref="A1:J73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4480,7 +4532,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
         <v>677.4299999999999</v>

</xml_diff>